<commit_message>
data: edita base de mapeamento Ingrooves via app
</commit_message>
<xml_diff>
--- a/data/mapping/mapping-artistas-ingrooves.xlsx
+++ b/data/mapping/mapping-artistas-ingrooves.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4302" uniqueCount="1664">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4302" uniqueCount="1663">
   <si>
     <t>Artist</t>
   </si>
@@ -4993,7 +4993,7 @@
     <t>NAS NUVENS PROJECTS - A BELEZA É VOCÊ MENINA</t>
   </si>
   <si>
-    <t>NAS NUVENS PROJECT - NETINHO &amp; FAMÍLIA DE PAULA - NA SEGUNDA ABSOLUTA, VOL. 1</t>
+    <t>NAS NUVENS PROJECT - NETINHO &amp; FAMÍLIA DE PAULA - NA SEGUNDA ABSOLUTA, VOL. 1 e 2</t>
   </si>
   <si>
     <t>CARLINHOS BROWN</t>
@@ -5003,9 +5003,6 @@
   </si>
   <si>
     <t>NAS NUVENS PROJECT - TANTINHO</t>
-  </si>
-  <si>
-    <t>NETINHO DE PAULA</t>
   </si>
 </sst>
 </file>
@@ -19063,7 +19060,7 @@
         <v>1603</v>
       </c>
       <c r="F685" t="s">
-        <v>1663</v>
+        <v>1659</v>
       </c>
     </row>
     <row r="686" spans="1:6">
@@ -19083,7 +19080,7 @@
         <v>1604</v>
       </c>
       <c r="F686" t="s">
-        <v>1663</v>
+        <v>1659</v>
       </c>
     </row>
     <row r="687" spans="1:6">
@@ -19103,7 +19100,7 @@
         <v>1605</v>
       </c>
       <c r="F687" t="s">
-        <v>1663</v>
+        <v>1659</v>
       </c>
     </row>
     <row r="688" spans="1:6">

</xml_diff>